<commit_message>
Update Trends in AI adoption costs (regions and sectors).xlsx
</commit_message>
<xml_diff>
--- a/Trends in AI adoption costs (regions and sectors).xlsx
+++ b/Trends in AI adoption costs (regions and sectors).xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Albert\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Albert\.spyder-py3\ITMO-3\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -2369,9 +2369,6 @@
     <t>93.29</t>
   </si>
   <si>
-    <t>Разница ((D/С)-1)</t>
-  </si>
-  <si>
     <t>Млн. руб, цены 24 года</t>
   </si>
   <si>
@@ -2772,6 +2769,9 @@
   </si>
   <si>
     <t>99</t>
+  </si>
+  <si>
+    <t>diff ((D/С)-1)</t>
   </si>
 </sst>
 </file>
@@ -3200,10 +3200,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>782</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>783</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>784</v>
       </c>
       <c r="C1" s="1">
         <v>2024</v>
@@ -3212,18 +3212,18 @@
         <v>2025</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>915</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>781</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>863</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>864</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>865</v>
       </c>
       <c r="C2" s="7">
         <v>90304.68</v>
@@ -3238,10 +3238,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>784</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>785</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>786</v>
       </c>
       <c r="C3" s="7">
         <v>74609.490000000005</v>
@@ -3256,10 +3256,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>786</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>787</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>788</v>
       </c>
       <c r="C4" s="7">
         <v>9050.1309999999994</v>
@@ -3274,10 +3274,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>789</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>790</v>
       </c>
       <c r="C5" s="7">
         <v>3019.8883999999998</v>
@@ -3292,10 +3292,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>790</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>791</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>792</v>
       </c>
       <c r="C6" s="7">
         <v>1329.3003000000001</v>
@@ -3310,10 +3310,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>793</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>794</v>
       </c>
       <c r="C7" s="7">
         <v>143.78469999999999</v>
@@ -3328,10 +3328,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>795</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>796</v>
       </c>
       <c r="C8" s="7">
         <v>555.11500000000001</v>
@@ -3346,10 +3346,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>796</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>797</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>798</v>
       </c>
       <c r="C9" s="7">
         <v>661.125</v>
@@ -3364,10 +3364,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>799</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>800</v>
       </c>
       <c r="C10" s="7">
         <v>935.83900000000006</v>
@@ -3382,10 +3382,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>801</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>802</v>
       </c>
       <c r="C11" s="7">
         <v>50.836399999999998</v>
@@ -3400,7 +3400,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>87</v>
@@ -3418,10 +3418,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>804</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>805</v>
       </c>
       <c r="C13" s="7">
         <v>29.985802</v>
@@ -3436,10 +3436,10 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>806</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>807</v>
       </c>
       <c r="C14" s="7">
         <v>25.970800000000001</v>
@@ -3454,10 +3454,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>808</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>809</v>
       </c>
       <c r="C15" s="7">
         <v>14.4567</v>
@@ -3472,7 +3472,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>115</v>
@@ -3490,10 +3490,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>811</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>812</v>
       </c>
       <c r="C17" s="7">
         <v>6.1675000000000004</v>
@@ -3508,7 +3508,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>119</v>
@@ -3526,7 +3526,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>123</v>
@@ -3544,7 +3544,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>127</v>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>131</v>
@@ -3580,7 +3580,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>143</v>
@@ -3598,7 +3598,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>157</v>
@@ -3616,7 +3616,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>163</v>
@@ -3634,7 +3634,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>187</v>
@@ -3652,7 +3652,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>189</v>
@@ -3670,7 +3670,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>199</v>
@@ -3688,10 +3688,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>822</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>823</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>824</v>
       </c>
       <c r="C28" s="7">
         <v>426.06220000000002</v>
@@ -3706,7 +3706,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>207</v>
@@ -3724,10 +3724,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>826</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>827</v>
       </c>
       <c r="C30" s="7">
         <v>56.112299999999998</v>
@@ -3742,7 +3742,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>209</v>
@@ -3760,10 +3760,10 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>829</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>830</v>
       </c>
       <c r="C32" s="7">
         <v>266.82641999999998</v>
@@ -3778,10 +3778,10 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>831</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>832</v>
       </c>
       <c r="C33" s="7">
         <v>1527.4745</v>
@@ -3796,10 +3796,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>832</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>833</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>834</v>
       </c>
       <c r="C34" s="7">
         <v>50.62</v>
@@ -3814,7 +3814,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>247</v>
@@ -3832,10 +3832,10 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>835</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>836</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>837</v>
       </c>
       <c r="C36" s="7">
         <v>104.9799</v>
@@ -3850,10 +3850,10 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>838</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>839</v>
       </c>
       <c r="C37" s="7">
         <v>8163.9224000000004</v>
@@ -3868,7 +3868,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>255</v>
@@ -3886,7 +3886,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>259</v>
@@ -3904,10 +3904,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>841</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>842</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>843</v>
       </c>
       <c r="C40" s="7">
         <v>3.1866998999999998</v>
@@ -3922,7 +3922,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>279</v>
@@ -3940,7 +3940,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>293</v>
@@ -3958,7 +3958,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>372</v>
@@ -3976,7 +3976,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>390</v>
@@ -3994,10 +3994,10 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
+        <v>847</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>848</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>849</v>
       </c>
       <c r="C45" s="7">
         <v>167.8305</v>
@@ -4012,7 +4012,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>412</v>
@@ -4030,7 +4030,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>414</v>
@@ -4048,10 +4048,10 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>851</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>852</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>853</v>
       </c>
       <c r="C48" s="7">
         <v>103.6416</v>
@@ -4066,10 +4066,10 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>853</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>854</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>855</v>
       </c>
       <c r="C49" s="7">
         <v>72.935294999999996</v>
@@ -4084,7 +4084,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>444</v>
@@ -4102,10 +4102,10 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
+        <v>856</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>857</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>858</v>
       </c>
       <c r="C51" s="7">
         <v>113.57559999999999</v>
@@ -4120,7 +4120,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>454</v>
@@ -4138,7 +4138,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>468</v>
@@ -4156,7 +4156,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>472</v>
@@ -4174,7 +4174,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>490</v>
@@ -4192,7 +4192,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>500</v>
@@ -4210,7 +4210,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>518</v>
@@ -4228,7 +4228,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>524</v>
@@ -4246,7 +4246,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>532</v>
@@ -4264,7 +4264,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>556</v>
@@ -4282,10 +4282,10 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
+        <v>869</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>870</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>871</v>
       </c>
       <c r="C61" s="7">
         <v>59.752299999999998</v>
@@ -4300,7 +4300,7 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>564</v>
@@ -4318,7 +4318,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>572</v>
@@ -4336,10 +4336,10 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
+        <v>873</v>
+      </c>
+      <c r="B64" s="2" t="s">
         <v>874</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>875</v>
       </c>
       <c r="C64" s="7">
         <v>796.61365000000001</v>
@@ -4354,10 +4354,10 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="B65" s="2" t="s">
         <v>876</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>877</v>
       </c>
       <c r="C65" s="7">
         <v>175.24680000000001</v>
@@ -4372,10 +4372,10 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
+        <v>877</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>878</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>879</v>
       </c>
       <c r="C66" s="7">
         <v>31.566198</v>
@@ -4390,7 +4390,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>604</v>
@@ -4408,10 +4408,10 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
+        <v>880</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>881</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>882</v>
       </c>
       <c r="C68" s="7">
         <v>226.81009</v>
@@ -4426,10 +4426,10 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>883</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>884</v>
       </c>
       <c r="C69" s="7">
         <v>278.38639999999998</v>
@@ -4444,7 +4444,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>618</v>
@@ -4462,10 +4462,10 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
+        <v>885</v>
+      </c>
+      <c r="B71" s="2" t="s">
         <v>886</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>887</v>
       </c>
       <c r="C71" s="7">
         <v>4.5687002999999997</v>
@@ -4480,10 +4480,10 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
+        <v>887</v>
+      </c>
+      <c r="B72" s="2" t="s">
         <v>888</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>889</v>
       </c>
       <c r="C72" s="7">
         <v>74.874700000000004</v>
@@ -4498,7 +4498,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>622</v>
@@ -4516,7 +4516,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>626</v>
@@ -4534,7 +4534,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>640</v>
@@ -4552,7 +4552,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>654</v>
@@ -4570,10 +4570,10 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
+        <v>893</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>894</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>895</v>
       </c>
       <c r="C77" s="7">
         <v>1.8684000000000001</v>
@@ -4588,7 +4588,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>712</v>
@@ -4606,7 +4606,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>736</v>
@@ -4624,10 +4624,10 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
+        <v>897</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>898</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>899</v>
       </c>
       <c r="C80" s="7">
         <v>23.8706</v>
@@ -4642,10 +4642,10 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>900</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>901</v>
       </c>
       <c r="C81" s="7">
         <v>4.7458996999999998</v>
@@ -4660,10 +4660,10 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
+        <v>901</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>902</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>903</v>
       </c>
       <c r="C82" s="7">
         <v>17.798400000000001</v>
@@ -4678,10 +4678,10 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>903</v>
+      </c>
+      <c r="B83" s="2" t="s">
         <v>904</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>905</v>
       </c>
       <c r="C83" s="7">
         <v>175.11199999999999</v>
@@ -4696,10 +4696,10 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
+        <v>905</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>906</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>907</v>
       </c>
       <c r="C84" s="7">
         <v>27.0503</v>
@@ -4714,10 +4714,10 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
+        <v>907</v>
+      </c>
+      <c r="B85" s="2" t="s">
         <v>908</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>909</v>
       </c>
       <c r="C85" s="7">
         <v>22.983301000000001</v>
@@ -4732,10 +4732,10 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
+        <v>909</v>
+      </c>
+      <c r="B86" s="2" t="s">
         <v>910</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>911</v>
       </c>
       <c r="C86" s="7">
         <v>20.080500000000001</v>
@@ -4750,10 +4750,10 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
+        <v>911</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>912</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>913</v>
       </c>
       <c r="C87" s="7">
         <v>105.9057</v>
@@ -4768,10 +4768,10 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
+        <v>913</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>914</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>915</v>
       </c>
       <c r="C88" s="7">
         <v>9.3339999999999996</v>
@@ -4817,10 +4817,10 @@
         <v>2025</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>915</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>781</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -4837,7 +4837,7 @@
         <v>166253.43025</v>
       </c>
       <c r="E2" s="5">
-        <f>(D2/C2)-1</f>
+        <f t="shared" ref="E2:E65" si="0">(D2/C2)-1</f>
         <v>0.84102791046258196</v>
       </c>
       <c r="G2" s="4"/>
@@ -4856,7 +4856,7 @@
         <v>3379.2858437499999</v>
       </c>
       <c r="E3" s="5">
-        <f>(D3/C3)-1</f>
+        <f t="shared" si="0"/>
         <v>-5.3513965958065679E-2</v>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
         <v>8780.2767499999991</v>
       </c>
       <c r="E4" s="5">
-        <f>(D4/C4)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.23405732059311313</v>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
         <v>70.378033325195304</v>
       </c>
       <c r="E5" s="5">
-        <f>(D5/C5)-1</f>
+        <f t="shared" si="0"/>
         <v>1.0123475850066281</v>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
         <v>5468.7938906250001</v>
       </c>
       <c r="E6" s="5">
-        <f>(D6/C6)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.38853305770050384</v>
       </c>
     </row>
@@ -4928,7 +4928,7 @@
         <v>63.830171264648428</v>
       </c>
       <c r="E7" s="5">
-        <f>(D7/C7)-1</f>
+        <f t="shared" si="0"/>
         <v>11.120036317221766</v>
       </c>
     </row>
@@ -4946,7 +4946,7 @@
         <v>85.039101196289053</v>
       </c>
       <c r="E8" s="5">
-        <f>(D8/C8)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.4365905870657677</v>
       </c>
     </row>
@@ -4964,7 +4964,7 @@
         <v>52.994744201660147</v>
       </c>
       <c r="E9" s="5">
-        <f>(D9/C9)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.24919288445264054</v>
       </c>
     </row>
@@ -4982,7 +4982,7 @@
         <v>115.77007800292969</v>
       </c>
       <c r="E10" s="5">
-        <f>(D10/C10)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.46126615629027434</v>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
         <v>97.741566406250001</v>
       </c>
       <c r="E11" s="5">
-        <f>(D11/C11)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.20730585301047011</v>
       </c>
     </row>
@@ -5018,7 +5018,7 @@
         <v>51.886960144042973</v>
       </c>
       <c r="E12" s="5">
-        <f>(D12/C12)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.17528474697539576</v>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
         <v>8.0938563385009754</v>
       </c>
       <c r="E13" s="5">
-        <f>(D13/C13)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.1153288514044184</v>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
         <v>6.7599837875366209</v>
       </c>
       <c r="E14" s="5">
-        <f>(D14/C14)-1</f>
+        <f t="shared" si="0"/>
         <v>-9.5218595238292569E-2</v>
       </c>
     </row>
@@ -5072,7 +5072,7 @@
         <v>43.793102905273443</v>
       </c>
       <c r="E15" s="5">
-        <f>(D15/C15)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.18548705677801125</v>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
         <v>11.814160324096679</v>
       </c>
       <c r="E16" s="5">
-        <f>(D16/C16)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.23309572709531456</v>
       </c>
     </row>
@@ -5108,7 +5108,7 @@
         <v>26.634016662597659</v>
       </c>
       <c r="E17" s="5">
-        <f>(D17/C17)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.26976073636394982</v>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
         <v>14.489362350463869</v>
       </c>
       <c r="E18" s="5">
-        <f>(D18/C18)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.48036442973981686</v>
       </c>
     </row>
@@ -5144,7 +5144,7 @@
         <v>14.404495834350589</v>
       </c>
       <c r="E19" s="5">
-        <f>(D19/C19)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.48340801850720716</v>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
         <v>30.685570861816409</v>
       </c>
       <c r="E20" s="5">
-        <f>(D20/C20)-1</f>
+        <f t="shared" si="0"/>
         <v>-3.707374833475352E-2</v>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
         <v>17.218275299072261</v>
       </c>
       <c r="E21" s="5">
-        <f>(D21/C21)-1</f>
+        <f t="shared" si="0"/>
         <v>-4.1079795550640119E-2</v>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
         <v>12.62411213684082</v>
       </c>
       <c r="E22" s="5">
-        <f>(D22/C22)-1</f>
+        <f t="shared" si="0"/>
         <v>0.27198929306083008</v>
       </c>
     </row>
@@ -5216,7 +5216,7 @@
         <v>0.83638397884368887</v>
       </c>
       <c r="E23" s="5">
-        <f>(D23/C23)-1</f>
+        <f t="shared" si="0"/>
         <v>1.5041436492326015</v>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
         <v>4.5941649627685548</v>
       </c>
       <c r="E24" s="5">
-        <f>(D24/C24)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.42796033434996583</v>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
         <v>3.9796209411621088</v>
       </c>
       <c r="E25" s="5">
-        <f>(D25/C25)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.50287051651899906</v>
       </c>
     </row>
@@ -5270,7 +5270,7 @@
         <v>3.914767845153809</v>
       </c>
       <c r="E26" s="5">
-        <f>(D26/C26)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.13543112960384063</v>
       </c>
     </row>
@@ -5288,7 +5288,7 @@
         <v>3.914767845153809</v>
       </c>
       <c r="E27" s="5">
-        <f>(D27/C27)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.13543112960384063</v>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
         <v>3.914767845153809</v>
       </c>
       <c r="E28" s="5">
-        <f>(D28/C28)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.13543112960384063</v>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
         <v>5.4933248367309568</v>
       </c>
       <c r="E29" s="5">
-        <f>(D29/C29)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.41455117853044765</v>
       </c>
     </row>
@@ -5342,7 +5342,7 @@
         <v>4.9786561584472651</v>
       </c>
       <c r="E30" s="5">
-        <f>(D30/C30)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.269134445324829</v>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
         <v>0.67968002700805663</v>
       </c>
       <c r="E31" s="5">
-        <f>(D31/C31)-1</f>
+        <f t="shared" si="0"/>
         <v>6.6499336274998599E-2</v>
       </c>
     </row>
@@ -5378,7 +5378,7 @@
         <v>0.67968002700805663</v>
       </c>
       <c r="E32" s="5">
-        <f>(D32/C32)-1</f>
+        <f t="shared" si="0"/>
         <v>6.6499336274998599E-2</v>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
         <v>9.5325115966796865</v>
       </c>
       <c r="E33" s="5">
-        <f>(D33/C33)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.88164971839707185</v>
       </c>
     </row>
@@ -5414,7 +5414,7 @@
         <v>2.0564094123840331</v>
       </c>
       <c r="E34" s="5">
-        <f>(D34/C34)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.597689638582797</v>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
         <v>6.9377391128540031</v>
       </c>
       <c r="E35" s="5">
-        <f>(D35/C35)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.90621876110495159</v>
       </c>
     </row>
@@ -5450,7 +5450,7 @@
         <v>0.53836318397521965</v>
       </c>
       <c r="E36" s="5">
-        <f>(D36/C36)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.63011804604931665</v>
       </c>
     </row>
@@ -5468,7 +5468,7 @@
         <v>974.81908789062493</v>
       </c>
       <c r="E37" s="5">
-        <f>(D37/C37)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.2439487903296329</v>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
         <v>797.90925878906251</v>
       </c>
       <c r="E38" s="5">
-        <f>(D38/C38)-1</f>
+        <f t="shared" si="0"/>
         <v>-5.2962216741707424E-2</v>
       </c>
     </row>
@@ -5504,7 +5504,7 @@
         <v>772.41935742187491</v>
       </c>
       <c r="E39" s="5">
-        <f>(D39/C39)-1</f>
+        <f t="shared" si="0"/>
         <v>-8.3216157801232704E-2</v>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
         <v>772.41935742187491</v>
       </c>
       <c r="E40" s="5">
-        <f>(D40/C40)-1</f>
+        <f t="shared" si="0"/>
         <v>-8.3216157801232704E-2</v>
       </c>
     </row>
@@ -5540,7 +5540,7 @@
         <v>772.41935742187491</v>
       </c>
       <c r="E41" s="5">
-        <f>(D41/C41)-1</f>
+        <f t="shared" si="0"/>
         <v>-8.3216157801232704E-2</v>
       </c>
     </row>
@@ -5558,7 +5558,7 @@
         <v>96.527968383789059</v>
       </c>
       <c r="E42" s="5">
-        <f>(D42/C42)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.73633542951819075</v>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
         <v>3034.8950078124999</v>
       </c>
       <c r="E43" s="5">
-        <f>(D43/C43)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.2663294998922181</v>
       </c>
     </row>
@@ -5594,7 +5594,7 @@
         <v>137.0565246582031</v>
       </c>
       <c r="E44" s="5">
-        <f>(D44/C44)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.32289578002989339</v>
       </c>
     </row>
@@ -5612,7 +5612,7 @@
         <v>35.758436523437503</v>
       </c>
       <c r="E45" s="5">
-        <f>(D45/C45)-1</f>
+        <f t="shared" si="0"/>
         <v>1.0704562917431444</v>
       </c>
     </row>
@@ -5630,7 +5630,7 @@
         <v>31.78674334716797</v>
       </c>
       <c r="E46" s="5">
-        <f>(D46/C46)-1</f>
+        <f t="shared" si="0"/>
         <v>1.4592273681612293</v>
       </c>
     </row>
@@ -5648,7 +5648,7 @@
         <v>47.446857238769532</v>
       </c>
       <c r="E47" s="5">
-        <f>(D47/C47)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.47984804155824023</v>
       </c>
     </row>
@@ -5666,7 +5666,7 @@
         <v>47.446857238769532</v>
       </c>
       <c r="E48" s="5">
-        <f>(D48/C48)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.47984804155824023</v>
       </c>
     </row>
@@ -5684,7 +5684,7 @@
         <v>6.7447854537963856</v>
       </c>
       <c r="E49" s="5">
-        <f>(D49/C49)-1</f>
+        <f t="shared" si="0"/>
         <v>0.13392042194216502</v>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
         <v>6.7447854537963856</v>
       </c>
       <c r="E50" s="5">
-        <f>(D50/C50)-1</f>
+        <f t="shared" si="0"/>
         <v>0.13392042194216502</v>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
         <v>7.8481325378417974</v>
       </c>
       <c r="E51" s="5">
-        <f>(D51/C51)-1</f>
+        <f t="shared" si="0"/>
         <v>2.7071953414462908</v>
       </c>
     </row>
@@ -5738,7 +5738,7 @@
         <v>7.3544207611083969</v>
       </c>
       <c r="E52" s="5">
-        <f>(D52/C52)-1</f>
+        <f t="shared" si="0"/>
         <v>2.6589158015464665</v>
       </c>
     </row>
@@ -5756,7 +5756,7 @@
         <v>5.7845491104125966</v>
       </c>
       <c r="E53" s="5">
-        <f>(D53/C53)-1</f>
+        <f t="shared" si="0"/>
         <v>1.8778851295585062</v>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
         <v>2.0352639045715328</v>
       </c>
       <c r="E54" s="5">
-        <f>(D54/C54)-1</f>
+        <f t="shared" si="0"/>
         <v>0.7540842063014157</v>
       </c>
     </row>
@@ -5792,7 +5792,7 @@
         <v>0.78068802070617671</v>
       </c>
       <c r="E55" s="5">
-        <f>(D55/C55)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.32716709410826805</v>
       </c>
     </row>
@@ -5810,7 +5810,7 @@
         <v>3.829902679443359</v>
       </c>
       <c r="E56" s="5">
-        <f>(D56/C56)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.53118349436997547</v>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
         <v>1.5400415897369379</v>
       </c>
       <c r="E57" s="5">
-        <f>(D57/C57)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.80486041691118371</v>
       </c>
     </row>
@@ -5846,7 +5846,7 @@
         <v>3.250947174072266</v>
       </c>
       <c r="E58" s="5">
-        <f>(D58/C58)-1</f>
+        <f t="shared" si="0"/>
         <v>1.2119801143582132</v>
       </c>
     </row>
@@ -5864,7 +5864,7 @@
         <v>5.5681839675903317</v>
       </c>
       <c r="E59" s="5">
-        <f>(D59/C59)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.26584692892210016</v>
       </c>
     </row>
@@ -5882,7 +5882,7 @@
         <v>24.54437811279297</v>
       </c>
       <c r="E60" s="5">
-        <f>(D60/C60)-1</f>
+        <f t="shared" si="0"/>
         <v>5.0994975429405986</v>
       </c>
     </row>
@@ -5900,7 +5900,7 @@
         <v>24.527858184814459</v>
       </c>
       <c r="E61" s="5">
-        <f>(D61/C61)-1</f>
+        <f t="shared" si="0"/>
         <v>5.0953921930453427</v>
       </c>
     </row>
@@ -5918,7 +5918,7 @@
         <v>2.8631519927978508</v>
       </c>
       <c r="E62" s="5">
-        <f>(D62/C62)-1</f>
+        <f t="shared" si="0"/>
         <v>1.1706990089445419</v>
       </c>
     </row>
@@ -5936,7 +5936,7 @@
         <v>2.8631519927978508</v>
       </c>
       <c r="E63" s="5">
-        <f>(D63/C63)-1</f>
+        <f t="shared" si="0"/>
         <v>1.1706990089445419</v>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
         <v>1756.6416855468749</v>
       </c>
       <c r="E64" s="5">
-        <f>(D64/C64)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.14888846941457745</v>
       </c>
     </row>
@@ -5972,7 +5972,7 @@
         <v>1756.6416855468749</v>
       </c>
       <c r="E65" s="5">
-        <f>(D65/C65)-1</f>
+        <f t="shared" si="0"/>
         <v>-0.14520886459226101</v>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
         <v>281.91749902343747</v>
       </c>
       <c r="E66" s="5">
-        <f>(D66/C66)-1</f>
+        <f t="shared" ref="E66:E129" si="1">(D66/C66)-1</f>
         <v>-0.39043929317955484</v>
       </c>
     </row>
@@ -6008,7 +6008,7 @@
         <v>250.10477392578119</v>
       </c>
       <c r="E67" s="5">
-        <f>(D67/C67)-1</f>
+        <f t="shared" si="1"/>
         <v>6.4964538142064931E-4</v>
       </c>
     </row>
@@ -6026,7 +6026,7 @@
         <v>224.23020581054689</v>
       </c>
       <c r="E68" s="5">
-        <f>(D68/C68)-1</f>
+        <f t="shared" si="1"/>
         <v>2.6520904203590767E-3</v>
       </c>
     </row>
@@ -6044,7 +6044,7 @@
         <v>31.04910290527344</v>
       </c>
       <c r="E69" s="5">
-        <f>(D69/C69)-1</f>
+        <f t="shared" si="1"/>
         <v>1.1772037658841206</v>
       </c>
     </row>
@@ -6062,7 +6062,7 @@
         <v>18.222031524658199</v>
       </c>
       <c r="E70" s="5">
-        <f>(D70/C70)-1</f>
+        <f t="shared" si="1"/>
         <v>0.15045340770618076</v>
       </c>
     </row>
@@ -6080,7 +6080,7 @@
         <v>18.222031524658199</v>
       </c>
       <c r="E71" s="5">
-        <f>(D71/C71)-1</f>
+        <f t="shared" si="1"/>
         <v>0.15045340770618076</v>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
         <v>8.2626431884765612</v>
       </c>
       <c r="E72" s="5">
-        <f>(D72/C72)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.59113233037040858</v>
       </c>
     </row>
@@ -6116,7 +6116,7 @@
         <v>2.5316193199157708</v>
       </c>
       <c r="E73" s="5">
-        <f>(D73/C73)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.78116459036393593</v>
       </c>
     </row>
@@ -6134,7 +6134,7 @@
         <v>1.3331167755126949</v>
       </c>
       <c r="E74" s="5">
-        <f>(D74/C74)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.86943028643362441</v>
       </c>
     </row>
@@ -6152,7 +6152,7 @@
         <v>44.941575500488277</v>
       </c>
       <c r="E75" s="5">
-        <f>(D75/C75)-1</f>
+        <f t="shared" si="1"/>
         <v>0.25643222382631659</v>
       </c>
     </row>
@@ -6170,7 +6170,7 @@
         <v>14.666266921997069</v>
       </c>
       <c r="E76" s="5">
-        <f>(D76/C76)-1</f>
+        <f t="shared" si="1"/>
         <v>0.73278200874256472</v>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
         <v>2.176863994598389</v>
       </c>
       <c r="E77" s="5">
-        <f>(D77/C77)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.6876540312511279</v>
       </c>
     </row>
@@ -6206,7 +6206,7 @@
         <v>1.8936640396118161</v>
       </c>
       <c r="E78" s="5">
-        <f>(D78/C78)-1</f>
+        <f t="shared" si="1"/>
         <v>0.32239108911439684</v>
       </c>
     </row>
@@ -6224,7 +6224,7 @@
         <v>191.66201855468751</v>
       </c>
       <c r="E79" s="5">
-        <f>(D79/C79)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.50955239756726756</v>
       </c>
     </row>
@@ -6242,7 +6242,7 @@
         <v>43.586743347167967</v>
       </c>
       <c r="E80" s="5">
-        <f>(D80/C80)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.67021013589683243</v>
       </c>
     </row>
@@ -6260,7 +6260,7 @@
         <v>95.176816528320302</v>
       </c>
       <c r="E81" s="5">
-        <f>(D81/C81)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.25848477047302354</v>
       </c>
     </row>
@@ -6278,7 +6278,7 @@
         <v>201.0289599609375</v>
       </c>
       <c r="E82" s="5">
-        <f>(D82/C82)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.60477745401100469</v>
       </c>
     </row>
@@ -6296,7 +6296,7 @@
         <v>179.6145959472656</v>
       </c>
       <c r="E83" s="5">
-        <f>(D83/C83)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.61833671664236367</v>
       </c>
     </row>
@@ -6314,7 +6314,7 @@
         <v>9.3780741271972659</v>
       </c>
       <c r="E84" s="5">
-        <f>(D84/C84)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.71048893188618256</v>
       </c>
     </row>
@@ -6332,7 +6332,7 @@
         <v>9.3780741271972659</v>
       </c>
       <c r="E85" s="5">
-        <f>(D85/C85)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.71048893188618256</v>
       </c>
     </row>
@@ -6350,7 +6350,7 @@
         <v>2.9814353523254389</v>
       </c>
       <c r="E86" s="5">
-        <f>(D86/C86)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.41386479134875187</v>
       </c>
     </row>
@@ -6368,7 +6368,7 @@
         <v>2.8211441116333011</v>
       </c>
       <c r="E87" s="5">
-        <f>(D87/C87)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.42719049123199504</v>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
         <v>143.61686083984381</v>
       </c>
       <c r="E88" s="5">
-        <f>(D88/C88)-1</f>
+        <f t="shared" si="1"/>
         <v>0.5711457388205079</v>
       </c>
     </row>
@@ -6404,7 +6404,7 @@
         <v>5.2760162124633787</v>
       </c>
       <c r="E89" s="5">
-        <f>(D89/C89)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.71139345700654344</v>
       </c>
     </row>
@@ -6422,7 +6422,7 @@
         <v>5.2760162124633787</v>
       </c>
       <c r="E90" s="5">
-        <f>(D90/C90)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.71139345700654344</v>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
         <v>63.644010131835927</v>
       </c>
       <c r="E91" s="5">
-        <f>(D91/C91)-1</f>
+        <f t="shared" si="1"/>
         <v>0.56735482765689604</v>
       </c>
     </row>
@@ -6458,7 +6458,7 @@
         <v>63.644010131835927</v>
       </c>
       <c r="E92" s="5">
-        <f>(D92/C92)-1</f>
+        <f t="shared" si="1"/>
         <v>0.56735482765689604</v>
       </c>
     </row>
@@ -6476,7 +6476,7 @@
         <v>51.379655212402341</v>
       </c>
       <c r="E93" s="5">
-        <f>(D93/C93)-1</f>
+        <f t="shared" si="1"/>
         <v>10.036334488755738</v>
       </c>
     </row>
@@ -6494,7 +6494,7 @@
         <v>22.062789642333978</v>
       </c>
       <c r="E94" s="5">
-        <f>(D94/C94)-1</f>
+        <f t="shared" si="1"/>
         <v>1.4075501573913116</v>
       </c>
     </row>
@@ -6512,7 +6512,7 @@
         <v>41.286125061035158</v>
       </c>
       <c r="E95" s="5">
-        <f>(D95/C95)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.73288239083294193</v>
       </c>
     </row>
@@ -6530,7 +6530,7 @@
         <v>10.579407791137699</v>
       </c>
       <c r="E96" s="5">
-        <f>(D96/C96)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.87289559805923422</v>
       </c>
     </row>
@@ -6548,7 +6548,7 @@
         <v>22.268299346923829</v>
       </c>
       <c r="E97" s="5">
-        <f>(D97/C97)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.32129949384874712</v>
       </c>
     </row>
@@ -6566,7 +6566,7 @@
         <v>18.8743355102539</v>
       </c>
       <c r="E98" s="5">
-        <f>(D98/C98)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.33283131578235925</v>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
         <v>18.8743355102539</v>
       </c>
       <c r="E99" s="5">
-        <f>(D99/C99)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.33283131578235925</v>
       </c>
     </row>
@@ -6602,7 +6602,7 @@
         <v>13.386298400878911</v>
       </c>
       <c r="E100" s="5">
-        <f>(D100/C100)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.82563158099263889</v>
       </c>
     </row>
@@ -6620,7 +6620,7 @@
         <v>1.1375200405120851</v>
       </c>
       <c r="E101" s="5">
-        <f>(D101/C101)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.7655564632085563</v>
       </c>
     </row>
@@ -6638,7 +6638,7 @@
         <v>1.8408000450134281</v>
       </c>
       <c r="E102" s="5">
-        <f>(D102/C102)-1</f>
+        <f t="shared" si="1"/>
         <v>0.17099239504670982</v>
       </c>
     </row>
@@ -6656,7 +6656,7 @@
         <v>1.2281439990997309</v>
       </c>
       <c r="E103" s="5">
-        <f>(D103/C103)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.11517002946705257</v>
       </c>
     </row>
@@ -6674,7 +6674,7 @@
         <v>118.03436145019531</v>
       </c>
       <c r="E104" s="5">
-        <f>(D104/C104)-1</f>
+        <f t="shared" si="1"/>
         <v>1.4622141680075278</v>
       </c>
     </row>
@@ -6692,7 +6692,7 @@
         <v>2.652639945983887</v>
       </c>
       <c r="E105" s="5">
-        <f>(D105/C105)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.73627877457037461</v>
       </c>
     </row>
@@ -6710,7 +6710,7 @@
         <v>2.652639945983887</v>
       </c>
       <c r="E106" s="5">
-        <f>(D106/C106)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.73588490606024926</v>
       </c>
     </row>
@@ -6728,7 +6728,7 @@
         <v>2.1466559333801269</v>
       </c>
       <c r="E107" s="5">
-        <f>(D107/C107)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.18819501063414623</v>
       </c>
     </row>
@@ -6746,7 +6746,7 @@
         <v>227.51334838867189</v>
       </c>
       <c r="E108" s="5">
-        <f>(D108/C108)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.46125809009397734</v>
       </c>
     </row>
@@ -6764,7 +6764,7 @@
         <v>227.51334838867189</v>
       </c>
       <c r="E109" s="5">
-        <f>(D109/C109)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.46125809009397734</v>
       </c>
     </row>
@@ -6782,7 +6782,7 @@
         <v>181.4525698242187</v>
       </c>
       <c r="E110" s="5">
-        <f>(D110/C110)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.50264838431066672</v>
       </c>
     </row>
@@ -6800,7 +6800,7 @@
         <v>56.608847106933588</v>
       </c>
       <c r="E111" s="5">
-        <f>(D111/C111)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.23203608721223024</v>
       </c>
     </row>
@@ -6818,7 +6818,7 @@
         <v>40.730767395019527</v>
       </c>
       <c r="E112" s="5">
-        <f>(D112/C112)-1</f>
+        <f t="shared" si="1"/>
         <v>-4.0090889283309727E-2</v>
       </c>
     </row>
@@ -6836,7 +6836,7 @@
         <v>39.312030578613268</v>
       </c>
       <c r="E113" s="5">
-        <f>(D113/C113)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.41698889683545182</v>
       </c>
     </row>
@@ -6854,7 +6854,7 @@
         <v>35.498835083007798</v>
       </c>
       <c r="E114" s="5">
-        <f>(D114/C114)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.28509906066973723</v>
       </c>
     </row>
@@ -6872,7 +6872,7 @@
         <v>1.4985999774932861</v>
       </c>
       <c r="E115" s="5">
-        <f>(D115/C115)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.96828735689540957</v>
       </c>
     </row>
@@ -6890,7 +6890,7 @@
         <v>10.56194438171387</v>
       </c>
       <c r="E116" s="5">
-        <f>(D116/C116)-1</f>
+        <f t="shared" si="1"/>
         <v>0.35206733255422895</v>
       </c>
     </row>
@@ -6908,7 +6908,7 @@
         <v>7.7120083312988266</v>
       </c>
       <c r="E117" s="5">
-        <f>(D117/C117)-1</f>
+        <f t="shared" si="1"/>
         <v>0.21168449908068365</v>
       </c>
     </row>
@@ -6926,7 +6926,7 @@
         <v>7.7120083312988266</v>
       </c>
       <c r="E118" s="5">
-        <f>(D118/C118)-1</f>
+        <f t="shared" si="1"/>
         <v>0.21168449908068365</v>
       </c>
     </row>
@@ -6944,7 +6944,7 @@
         <v>212.42728173828129</v>
       </c>
       <c r="E119" s="5">
-        <f>(D119/C119)-1</f>
+        <f t="shared" si="1"/>
         <v>-7.0922372769969599E-2</v>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
         <v>182.23155419921869</v>
       </c>
       <c r="E120" s="5">
-        <f>(D120/C120)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.10779533275029218</v>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
         <v>30.90089709472656</v>
       </c>
       <c r="E121" s="5">
-        <f>(D121/C121)-1</f>
+        <f t="shared" si="1"/>
         <v>1.9149314770186079</v>
       </c>
     </row>
@@ -6998,7 +6998,7 @@
         <v>1.461595226287842</v>
       </c>
       <c r="E122" s="5">
-        <f>(D122/C122)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.22334065237906264</v>
       </c>
     </row>
@@ -7016,7 +7016,7 @@
         <v>1.8637392253875731</v>
       </c>
       <c r="E123" s="5">
-        <f>(D123/C123)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.91126572466683931</v>
       </c>
     </row>
@@ -7034,7 +7034,7 @@
         <v>4.7319888763427729</v>
       </c>
       <c r="E124" s="5">
-        <f>(D124/C124)-1</f>
+        <f t="shared" si="1"/>
         <v>0.39545528644729377</v>
       </c>
     </row>
@@ -7052,7 +7052,7 @@
         <v>4.522420761108398</v>
       </c>
       <c r="E125" s="5">
-        <f>(D125/C125)-1</f>
+        <f t="shared" si="1"/>
         <v>0.67652298836270552</v>
       </c>
     </row>
@@ -7070,7 +7070,7 @@
         <v>4.522420761108398</v>
       </c>
       <c r="E126" s="5">
-        <f>(D126/C126)-1</f>
+        <f t="shared" si="1"/>
         <v>0.72776342353711465</v>
       </c>
     </row>
@@ -7088,7 +7088,7 @@
         <v>137.71638549804689</v>
       </c>
       <c r="E127" s="5">
-        <f>(D127/C127)-1</f>
+        <f t="shared" si="1"/>
         <v>4.1494473317877922E-3</v>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
         <v>15.825594055175779</v>
       </c>
       <c r="E128" s="5">
-        <f>(D128/C128)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.80662338547065082</v>
       </c>
     </row>
@@ -7124,7 +7124,7 @@
         <v>15.825594055175779</v>
       </c>
       <c r="E129" s="5">
-        <f>(D129/C129)-1</f>
+        <f t="shared" si="1"/>
         <v>-0.80662338547065082</v>
       </c>
     </row>
@@ -7142,7 +7142,7 @@
         <v>95.678172485351567</v>
       </c>
       <c r="E130" s="5">
-        <f>(D130/C130)-1</f>
+        <f t="shared" ref="E130:E193" si="2">(D130/C130)-1</f>
         <v>1.3486452929321207</v>
       </c>
     </row>
@@ -7160,7 +7160,7 @@
         <v>18.247426300048829</v>
       </c>
       <c r="E131" s="5">
-        <f>(D131/C131)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.41067756447777604</v>
       </c>
     </row>
@@ -7178,7 +7178,7 @@
         <v>15.97993789672852</v>
       </c>
       <c r="E132" s="5">
-        <f>(D132/C132)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.42279436890993238</v>
       </c>
     </row>
@@ -7196,7 +7196,7 @@
         <v>24.57666174316406</v>
       </c>
       <c r="E133" s="5">
-        <f>(D133/C133)-1</f>
+        <f t="shared" si="2"/>
         <v>1.7953754868872553</v>
       </c>
     </row>
@@ -7214,7 +7214,7 @@
         <v>24.57666174316406</v>
       </c>
       <c r="E134" s="5">
-        <f>(D134/C134)-1</f>
+        <f t="shared" si="2"/>
         <v>7.5935388451218788</v>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
         <v>26.212613555908199</v>
       </c>
       <c r="E135" s="5">
-        <f>(D135/C135)-1</f>
+        <f t="shared" si="2"/>
         <v>0.79889603375824025</v>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
         <v>0.85583039855957033</v>
       </c>
       <c r="E136" s="5">
-        <f>(D136/C136)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.88909516916862297</v>
       </c>
     </row>
@@ -7268,7 +7268,7 @@
         <v>2.7848000450134269</v>
       </c>
       <c r="E137" s="5">
-        <f>(D137/C137)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.13110763026102124</v>
       </c>
     </row>
@@ -7286,7 +7286,7 @@
         <v>2.7848000450134269</v>
       </c>
       <c r="E138" s="5">
-        <f>(D138/C138)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.13110763026102124</v>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
         <v>1168.9430312500001</v>
       </c>
       <c r="E139" s="5">
-        <f>(D139/C139)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.27502742114500134</v>
       </c>
     </row>
@@ -7322,7 +7322,7 @@
         <v>43.396811889648433</v>
       </c>
       <c r="E140" s="5">
-        <f>(D140/C140)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.4627598113622462</v>
       </c>
     </row>
@@ -7340,7 +7340,7 @@
         <v>34.206027832031253</v>
       </c>
       <c r="E141" s="5">
-        <f>(D141/C141)-1</f>
+        <f t="shared" si="2"/>
         <v>-3.2295606150594236E-2</v>
       </c>
     </row>
@@ -7358,7 +7358,7 @@
         <v>34.000237243652343</v>
       </c>
       <c r="E142" s="5">
-        <f>(D142/C142)-1</f>
+        <f t="shared" si="2"/>
         <v>-3.7545723515641338E-2</v>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
         <v>10.82428173828125</v>
       </c>
       <c r="E143" s="5">
-        <f>(D143/C143)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.63591138392181412</v>
       </c>
     </row>
@@ -7394,7 +7394,7 @@
         <v>9.1615199279785173</v>
       </c>
       <c r="E144" s="5">
-        <f>(D144/C144)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.71156356581844371</v>
       </c>
     </row>
@@ -7412,7 +7412,7 @@
         <v>9.1615199279785173</v>
       </c>
       <c r="E145" s="5">
-        <f>(D145/C145)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.70964386794225165</v>
       </c>
     </row>
@@ -7430,7 +7430,7 @@
         <v>9.1615199279785173</v>
       </c>
       <c r="E146" s="5">
-        <f>(D146/C146)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.70583071606846592</v>
       </c>
     </row>
@@ -7448,7 +7448,7 @@
         <v>667.60055664062497</v>
       </c>
       <c r="E147" s="5">
-        <f>(D147/C147)-1</f>
+        <f t="shared" si="2"/>
         <v>0.63780810783182451</v>
       </c>
     </row>
@@ -7466,7 +7466,7 @@
         <v>26.559533843994139</v>
       </c>
       <c r="E148" s="5">
-        <f>(D148/C148)-1</f>
+        <f t="shared" si="2"/>
         <v>0.82261661547289622</v>
       </c>
     </row>
@@ -7484,7 +7484,7 @@
         <v>26.314943481445319</v>
       </c>
       <c r="E149" s="5">
-        <f>(D149/C149)-1</f>
+        <f t="shared" si="2"/>
         <v>1.5138463394579023</v>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
         <v>9.0208637695312515</v>
       </c>
       <c r="E150" s="5">
-        <f>(D150/C150)-1</f>
+        <f t="shared" si="2"/>
         <v>0.15015092940779939</v>
       </c>
     </row>
@@ -7520,7 +7520,7 @@
         <v>8.9914105834960925</v>
       </c>
       <c r="E151" s="5">
-        <f>(D151/C151)-1</f>
+        <f t="shared" si="2"/>
         <v>0.1499143881082583</v>
       </c>
     </row>
@@ -7538,7 +7538,7 @@
         <v>4.8510268859863279</v>
       </c>
       <c r="E152" s="5">
-        <f>(D152/C152)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.20472361618637858</v>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
         <v>122.3424921875</v>
       </c>
       <c r="E153" s="5">
-        <f>(D153/C153)-1</f>
+        <f t="shared" si="2"/>
         <v>1.8078558733920107</v>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
         <v>9.5976478271484371</v>
       </c>
       <c r="E154" s="5">
-        <f>(D154/C154)-1</f>
+        <f t="shared" si="2"/>
         <v>5.1912300213550644E-2</v>
       </c>
     </row>
@@ -7592,7 +7592,7 @@
         <v>2.70210542678833</v>
       </c>
       <c r="E155" s="5">
-        <f>(D155/C155)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.67383209082271134</v>
       </c>
     </row>
@@ -7610,7 +7610,7 @@
         <v>2.6945535240173339</v>
       </c>
       <c r="E156" s="5">
-        <f>(D156/C156)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.64680584551030473</v>
       </c>
     </row>
@@ -7628,7 +7628,7 @@
         <v>99.10658959960935</v>
       </c>
       <c r="E157" s="5">
-        <f>(D157/C157)-1</f>
+        <f t="shared" si="2"/>
         <v>4.7637870739012218</v>
       </c>
     </row>
@@ -7646,7 +7646,7 @@
         <v>93.716350463867187</v>
       </c>
       <c r="E158" s="5">
-        <f>(D158/C158)-1</f>
+        <f t="shared" si="2"/>
         <v>6.0512727293421111</v>
       </c>
     </row>
@@ -7664,7 +7664,7 @@
         <v>0.43886558771133422</v>
       </c>
       <c r="E159" s="5">
-        <f>(D159/C159)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.77498688078787215</v>
       </c>
     </row>
@@ -7682,7 +7682,7 @@
         <v>335.15200634765631</v>
       </c>
       <c r="E160" s="5">
-        <f>(D160/C160)-1</f>
+        <f t="shared" si="2"/>
         <v>0.89951964713102162</v>
       </c>
     </row>
@@ -7700,7 +7700,7 @@
         <v>5.9213345642089843</v>
       </c>
       <c r="E161" s="5">
-        <f>(D161/C161)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.56794978809437402</v>
       </c>
     </row>
@@ -7718,7 +7718,7 @@
         <v>7.838032424926757</v>
       </c>
       <c r="E162" s="5">
-        <f>(D162/C162)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.37467829134806951</v>
       </c>
     </row>
@@ -7736,7 +7736,7 @@
         <v>214.66758203124999</v>
       </c>
       <c r="E163" s="5">
-        <f>(D163/C163)-1</f>
+        <f t="shared" si="2"/>
         <v>6.4667504480465947</v>
       </c>
     </row>
@@ -7754,7 +7754,7 @@
         <v>176.39745385742191</v>
       </c>
       <c r="E164" s="5">
-        <f>(D164/C164)-1</f>
+        <f t="shared" si="2"/>
         <v>5.7450846534651996</v>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
         <v>93.240958251953117</v>
       </c>
       <c r="E165" s="5">
-        <f>(D165/C165)-1</f>
+        <f t="shared" si="2"/>
         <v>13.880459344390857</v>
       </c>
     </row>
@@ -7790,7 +7790,7 @@
         <v>4.8169490203857421</v>
       </c>
       <c r="E166" s="5">
-        <f>(D166/C166)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.93168901623220957</v>
       </c>
     </row>
@@ -7808,7 +7808,7 @@
         <v>4.8169490203857421</v>
       </c>
       <c r="E167" s="5">
-        <f>(D167/C167)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.93165315388652148</v>
       </c>
     </row>
@@ -7826,7 +7826,7 @@
         <v>66.388021484375003</v>
       </c>
       <c r="E168" s="5">
-        <f>(D168/C168)-1</f>
+        <f t="shared" si="2"/>
         <v>0.79383935983979548</v>
       </c>
     </row>
@@ -7844,7 +7844,7 @@
         <v>3.4201119117736809</v>
       </c>
       <c r="E169" s="5">
-        <f>(D169/C169)-1</f>
+        <f t="shared" si="2"/>
         <v>0.19413145901807916</v>
       </c>
     </row>
@@ -7862,7 +7862,7 @@
         <v>1.999392028808594</v>
       </c>
       <c r="E170" s="5">
-        <f>(D170/C170)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.17554243997831265</v>
       </c>
     </row>
@@ -7880,7 +7880,7 @@
         <v>53.656585632324223</v>
       </c>
       <c r="E171" s="5">
-        <f>(D171/C171)-1</f>
+        <f t="shared" si="2"/>
         <v>3.3682193555794182</v>
       </c>
     </row>
@@ -7898,7 +7898,7 @@
         <v>43.560502319335939</v>
       </c>
       <c r="E172" s="5">
-        <f>(D172/C172)-1</f>
+        <f t="shared" si="2"/>
         <v>16.650122495679067</v>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
         <v>74.311868408203125</v>
       </c>
       <c r="E173" s="5">
-        <f>(D173/C173)-1</f>
+        <f t="shared" si="2"/>
         <v>0.47190688275357373</v>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
         <v>20.071516235351559</v>
       </c>
       <c r="E174" s="5">
-        <f>(D174/C174)-1</f>
+        <f t="shared" si="2"/>
         <v>1.2360567533785147</v>
       </c>
     </row>
@@ -7952,7 +7952,7 @@
         <v>8.4050926818847653</v>
       </c>
       <c r="E175" s="5">
-        <f>(D175/C175)-1</f>
+        <f t="shared" si="2"/>
         <v>0.27814669736690467</v>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
         <v>1.389945665359497</v>
       </c>
       <c r="E176" s="5">
-        <f>(D176/C176)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.24183403405907544</v>
       </c>
     </row>
@@ -7988,7 +7988,7 @@
         <v>21.53377203369141</v>
       </c>
       <c r="E177" s="5">
-        <f>(D177/C177)-1</f>
+        <f t="shared" si="2"/>
         <v>1.0353666452760364</v>
       </c>
     </row>
@@ -8006,7 +8006,7 @@
         <v>20.370291961669921</v>
       </c>
       <c r="E178" s="5">
-        <f>(D178/C178)-1</f>
+        <f t="shared" si="2"/>
         <v>0.99742035061431045</v>
       </c>
     </row>
@@ -8024,7 +8024,7 @@
         <v>0.98940639495849603</v>
       </c>
       <c r="E179" s="5">
-        <f>(D179/C179)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.84646798023703185</v>
       </c>
     </row>
@@ -8042,7 +8042,7 @@
         <v>23.973352172851559</v>
       </c>
       <c r="E180" s="5">
-        <f>(D180/C180)-1</f>
+        <f t="shared" si="2"/>
         <v>-1.8398777659654364E-2</v>
       </c>
     </row>
@@ -8060,7 +8060,7 @@
         <v>18.591892456054691</v>
       </c>
       <c r="E181" s="5">
-        <f>(D181/C181)-1</f>
+        <f t="shared" si="2"/>
         <v>2.2480027351120158</v>
       </c>
     </row>
@@ -8078,7 +8078,7 @@
         <v>5.2923470840454101</v>
       </c>
       <c r="E182" s="5">
-        <f>(D182/C182)-1</f>
+        <f t="shared" si="2"/>
         <v>0.39455786140854032</v>
       </c>
     </row>
@@ -8096,7 +8096,7 @@
         <v>4.6520319747924814</v>
       </c>
       <c r="E183" s="5">
-        <f>(D183/C183)-1</f>
+        <f t="shared" si="2"/>
         <v>0.28829464823940221</v>
       </c>
     </row>
@@ -8114,7 +8114,7 @@
         <v>0.64031516551971435</v>
       </c>
       <c r="E184" s="5">
-        <f>(D184/C184)-1</f>
+        <f t="shared" si="2"/>
         <v>2.4799737256506216</v>
       </c>
     </row>
@@ -8132,7 +8132,7 @@
         <v>0.88924797344207751</v>
       </c>
       <c r="E185" s="5">
-        <f>(D185/C185)-1</f>
+        <f t="shared" si="2"/>
         <v>2.3430374941431484</v>
       </c>
     </row>
@@ -8150,7 +8150,7 @@
         <v>29.00883688354492</v>
       </c>
       <c r="E186" s="5">
-        <f>(D186/C186)-1</f>
+        <f t="shared" si="2"/>
         <v>3.0400591735087561</v>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
         <v>457.94564111328123</v>
       </c>
       <c r="E187" s="5">
-        <f>(D187/C187)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.59257526987682996</v>
       </c>
     </row>
@@ -8186,7 +8186,7 @@
         <v>259.77385986328119</v>
       </c>
       <c r="E188" s="5">
-        <f>(D188/C188)-1</f>
+        <f t="shared" si="2"/>
         <v>3.8285373313100477</v>
       </c>
     </row>
@@ -8204,7 +8204,7 @@
         <v>257.29776123046872</v>
       </c>
       <c r="E189" s="5">
-        <f>(D189/C189)-1</f>
+        <f t="shared" si="2"/>
         <v>4.0005881277360862</v>
       </c>
     </row>
@@ -8222,7 +8222,7 @@
         <v>36.690448547363282</v>
       </c>
       <c r="E190" s="5">
-        <f>(D190/C190)-1</f>
+        <f t="shared" si="2"/>
         <v>3.4454572164610786E-2</v>
       </c>
     </row>
@@ -8240,7 +8240,7 @@
         <v>1.9569119567871089</v>
       </c>
       <c r="E191" s="5">
-        <f>(D191/C191)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.23736868402684763</v>
       </c>
     </row>
@@ -8258,7 +8258,7 @@
         <v>105.8787625732422</v>
       </c>
       <c r="E192" s="5">
-        <f>(D192/C192)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.89292158439755587</v>
       </c>
     </row>
@@ -8276,7 +8276,7 @@
         <v>64.457831298828125</v>
       </c>
       <c r="E193" s="5">
-        <f>(D193/C193)-1</f>
+        <f t="shared" si="2"/>
         <v>-0.93444450753534369</v>
       </c>
     </row>
@@ -8294,7 +8294,7 @@
         <v>4.6158771896362314</v>
       </c>
       <c r="E194" s="5">
-        <f>(D194/C194)-1</f>
+        <f t="shared" ref="E194:E257" si="3">(D194/C194)-1</f>
         <v>3.2770799939645379E-3</v>
       </c>
     </row>
@@ -8312,7 +8312,7 @@
         <v>3132.0207617187498</v>
       </c>
       <c r="E195" s="5">
-        <f>(D195/C195)-1</f>
+        <f t="shared" si="3"/>
         <v>0.67389697452542907</v>
       </c>
     </row>
@@ -8330,7 +8330,7 @@
         <v>2861.5613046875001</v>
       </c>
       <c r="E196" s="5">
-        <f>(D196/C196)-1</f>
+        <f t="shared" si="3"/>
         <v>1.2594960004165152</v>
       </c>
     </row>
@@ -8348,7 +8348,7 @@
         <v>862.18002148437483</v>
       </c>
       <c r="E197" s="5">
-        <f>(D197/C197)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.13797100599537482</v>
       </c>
     </row>
@@ -8366,7 +8366,7 @@
         <v>1727.4729843749999</v>
       </c>
       <c r="E198" s="5">
-        <f>(D198/C198)-1</f>
+        <f t="shared" si="3"/>
         <v>143.37597549330971</v>
       </c>
     </row>
@@ -8384,7 +8384,7 @@
         <v>1727.0614824218751</v>
       </c>
       <c r="E199" s="5">
-        <f>(D199/C199)-1</f>
+        <f t="shared" si="3"/>
         <v>149.8179405326797</v>
       </c>
     </row>
@@ -8402,7 +8402,7 @@
         <v>3.6515808601379391</v>
       </c>
       <c r="E200" s="5">
-        <f>(D200/C200)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.20858672298700931</v>
       </c>
     </row>
@@ -8420,7 +8420,7 @@
         <v>3.6515808601379391</v>
       </c>
       <c r="E201" s="5">
-        <f>(D201/C201)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.20858672298700931</v>
       </c>
     </row>
@@ -8438,7 +8438,7 @@
         <v>1720.3720117187499</v>
       </c>
       <c r="E202" s="5">
-        <f>(D202/C202)-1</f>
+        <f t="shared" si="3"/>
         <v>401.96348621993064</v>
       </c>
     </row>
@@ -8456,7 +8456,7 @@
         <v>2.9736943931579591</v>
       </c>
       <c r="E203" s="5">
-        <f>(D203/C203)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.14632416800885373</v>
       </c>
     </row>
@@ -8474,7 +8474,7 @@
         <v>13.81572290039062</v>
       </c>
       <c r="E204" s="5">
-        <f>(D204/C204)-1</f>
+        <f t="shared" si="3"/>
         <v>0.22250052210301741</v>
       </c>
     </row>
@@ -8492,7 +8492,7 @@
         <v>13.50797869873047</v>
       </c>
       <c r="E205" s="5">
-        <f>(D205/C205)-1</f>
+        <f t="shared" si="3"/>
         <v>0.195269413755218</v>
       </c>
     </row>
@@ -8510,7 +8510,7 @@
         <v>10.48047727966309</v>
       </c>
       <c r="E206" s="5">
-        <f>(D206/C206)-1</f>
+        <f t="shared" si="3"/>
         <v>1.1604776911282393</v>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
         <v>12.712754379272461</v>
       </c>
       <c r="E207" s="5">
-        <f>(D207/C207)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.36958526709846617</v>
       </c>
     </row>
@@ -8546,7 +8546,7 @@
         <v>120.3361176757812</v>
       </c>
       <c r="E208" s="5">
-        <f>(D208/C208)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.79098631505742378</v>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
         <v>85.293041748046875</v>
       </c>
       <c r="E209" s="5">
-        <f>(D209/C209)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.84207840706500925</v>
       </c>
     </row>
@@ -8582,7 +8582,7 @@
         <v>11.24549398803711</v>
       </c>
       <c r="E210" s="5">
-        <f>(D210/C210)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.5103416359820121</v>
       </c>
     </row>
@@ -8600,7 +8600,7 @@
         <v>10.89574235534668</v>
       </c>
       <c r="E211" s="5">
-        <f>(D211/C211)-1</f>
+        <f t="shared" si="3"/>
         <v>1.0160500241181758</v>
       </c>
     </row>
@@ -8618,7 +8618,7 @@
         <v>9.2488396759033193</v>
       </c>
       <c r="E212" s="5">
-        <f>(D212/C212)-1</f>
+        <f t="shared" si="3"/>
         <v>0.71132198647484879</v>
       </c>
     </row>
@@ -8636,7 +8636,7 @@
         <v>3.8395310516357419</v>
       </c>
       <c r="E213" s="5">
-        <f>(D213/C213)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.99019272862510865</v>
       </c>
     </row>
@@ -8654,7 +8654,7 @@
         <v>3.8395310516357419</v>
       </c>
       <c r="E214" s="5">
-        <f>(D214/C214)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.99019272862510865</v>
       </c>
     </row>
@@ -8672,7 +8672,7 @@
         <v>2.2328431434631351</v>
       </c>
       <c r="E215" s="5">
-        <f>(D215/C215)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.99427226446537431</v>
       </c>
     </row>
@@ -8690,7 +8690,7 @@
         <v>49.382056518554677</v>
       </c>
       <c r="E216" s="5">
-        <f>(D216/C216)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.49103780965158805</v>
       </c>
     </row>
@@ -8708,7 +8708,7 @@
         <v>48.904863769531246</v>
       </c>
       <c r="E217" s="5">
-        <f>(D217/C217)-1</f>
+        <f t="shared" si="3"/>
         <v>-3.8611654061781353E-2</v>
       </c>
     </row>
@@ -8726,7 +8726,7 @@
         <v>20.56069876098633</v>
       </c>
       <c r="E218" s="5">
-        <f>(D218/C218)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.28129548514449354</v>
       </c>
     </row>
@@ -8744,7 +8744,7 @@
         <v>42.517854492187503</v>
       </c>
       <c r="E219" s="5">
-        <f>(D219/C219)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.76647818206181006</v>
       </c>
     </row>
@@ -8762,7 +8762,7 @@
         <v>39.894288269042967</v>
       </c>
       <c r="E220" s="5">
-        <f>(D220/C220)-1</f>
+        <f t="shared" si="3"/>
         <v>5.2619548680787593</v>
       </c>
     </row>
@@ -8780,7 +8780,7 @@
         <v>34.745148254394529</v>
       </c>
       <c r="E221" s="5">
-        <f>(D221/C221)-1</f>
+        <f t="shared" si="3"/>
         <v>4.8515187871593062</v>
       </c>
     </row>
@@ -8798,7 +8798,7 @@
         <v>5.0602173385620111</v>
       </c>
       <c r="E222" s="5">
-        <f>(D222/C222)-1</f>
+        <f t="shared" si="3"/>
         <v>13.334893310373969</v>
       </c>
     </row>
@@ -8816,7 +8816,7 @@
         <v>2.6235646476745602</v>
       </c>
       <c r="E223" s="5">
-        <f>(D223/C223)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.9850680492718068</v>
       </c>
     </row>
@@ -8834,7 +8834,7 @@
         <v>1.620942422866821</v>
       </c>
       <c r="E224" s="5">
-        <f>(D224/C224)-1</f>
+        <f t="shared" si="3"/>
         <v>-8.3177362631888574E-2</v>
       </c>
     </row>
@@ -8852,7 +8852,7 @@
         <v>1.002622337341309</v>
       </c>
       <c r="E225" s="5">
-        <f>(D225/C225)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.99423559628374247</v>
       </c>
     </row>
@@ -8870,7 +8870,7 @@
         <v>1.002622337341309</v>
       </c>
       <c r="E226" s="5">
-        <f>(D226/C226)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.99423559628374247</v>
       </c>
     </row>
@@ -8888,7 +8888,7 @@
         <v>8765.866</v>
       </c>
       <c r="E227" s="5">
-        <f>(D227/C227)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.22951091776690247</v>
       </c>
     </row>
@@ -8906,7 +8906,7 @@
         <v>22.945241882324218</v>
       </c>
       <c r="E228" s="5">
-        <f>(D228/C228)-1</f>
+        <f t="shared" si="3"/>
         <v>6.2307194032471624</v>
       </c>
     </row>
@@ -8924,7 +8924,7 @@
         <v>14.56318167114258</v>
       </c>
       <c r="E229" s="5">
-        <f>(D229/C229)-1</f>
+        <f t="shared" si="3"/>
         <v>3.5892861283656075</v>
       </c>
     </row>
@@ -8942,7 +8942,7 @@
         <v>8.0765810852050777</v>
       </c>
       <c r="E230" s="5">
-        <f>(D230/C230)-1</f>
+        <f t="shared" si="3"/>
         <v>4.9946419395866384</v>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
         <v>7.1934689483642584</v>
       </c>
       <c r="E231" s="5">
-        <f>(D231/C231)-1</f>
+        <f t="shared" si="3"/>
         <v>15.487437424625849</v>
       </c>
     </row>
@@ -8978,7 +8978,7 @@
         <v>34.68992218017577</v>
       </c>
       <c r="E232" s="5">
-        <f>(D232/C232)-1</f>
+        <f t="shared" si="3"/>
         <v>6.8336883635200349</v>
       </c>
     </row>
@@ -8996,7 +8996,7 @@
         <v>34.68992218017577</v>
       </c>
       <c r="E233" s="5">
-        <f>(D233/C233)-1</f>
+        <f t="shared" si="3"/>
         <v>6.8336883635200349</v>
       </c>
     </row>
@@ -9014,7 +9014,7 @@
         <v>0.73462082862853995</v>
       </c>
       <c r="E234" s="5">
-        <f>(D234/C234)-1</f>
+        <f t="shared" si="3"/>
         <v>0.23777730181725354</v>
       </c>
     </row>
@@ -9032,7 +9032,7 @@
         <v>11.889396667480471</v>
       </c>
       <c r="E235" s="5">
-        <f>(D235/C235)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.5033980048250748</v>
       </c>
     </row>
@@ -9050,7 +9050,7 @@
         <v>11.889396667480471</v>
       </c>
       <c r="E236" s="5">
-        <f>(D236/C236)-1</f>
+        <f t="shared" si="3"/>
         <v>0.21143603389752408</v>
       </c>
     </row>
@@ -9068,7 +9068,7 @@
         <v>1708.1890878906249</v>
       </c>
       <c r="E237" s="5">
-        <f>(D237/C237)-1</f>
+        <f t="shared" si="3"/>
         <v>0.14521547538486668</v>
       </c>
     </row>
@@ -9086,7 +9086,7 @@
         <v>670.33005566406246</v>
       </c>
       <c r="E238" s="5">
-        <f>(D238/C238)-1</f>
+        <f t="shared" si="3"/>
         <v>0.24869381206922636</v>
       </c>
     </row>
@@ -9104,7 +9104,7 @@
         <v>129.19499072265631</v>
       </c>
       <c r="E239" s="5">
-        <f>(D239/C239)-1</f>
+        <f t="shared" si="3"/>
         <v>4.0814155643129322</v>
       </c>
     </row>
@@ -9122,7 +9122,7 @@
         <v>5127.8370390624996</v>
       </c>
       <c r="E240" s="5">
-        <f>(D240/C240)-1</f>
+        <f t="shared" si="3"/>
         <v>0.14004426906400003</v>
       </c>
     </row>
@@ -9140,7 +9140,7 @@
         <v>2998.1917070312502</v>
       </c>
       <c r="E241" s="5">
-        <f>(D241/C241)-1</f>
+        <f t="shared" si="3"/>
         <v>-7.3032340281595887E-2</v>
       </c>
     </row>
@@ -9158,7 +9158,7 @@
         <v>66.273708984374991</v>
       </c>
       <c r="E242" s="5">
-        <f>(D242/C242)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.77286886186704917</v>
       </c>
     </row>
@@ -9176,7 +9176,7 @@
         <v>45.231289123535163</v>
       </c>
       <c r="E243" s="5">
-        <f>(D243/C243)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.83520786198392294</v>
       </c>
     </row>
@@ -9194,7 +9194,7 @@
         <v>553.24928027343742</v>
       </c>
       <c r="E244" s="5">
-        <f>(D244/C244)-1</f>
+        <f t="shared" si="3"/>
         <v>7.5106108614985683</v>
       </c>
     </row>
@@ -9212,7 +9212,7 @@
         <v>1510.122515625</v>
       </c>
       <c r="E245" s="5">
-        <f>(D245/C245)-1</f>
+        <f t="shared" si="3"/>
         <v>0.66546584442524459</v>
       </c>
     </row>
@@ -9230,7 +9230,7 @@
         <v>1860.314826171875</v>
       </c>
       <c r="E246" s="5">
-        <f>(D246/C246)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.65266432028745813</v>
       </c>
     </row>
@@ -9248,7 +9248,7 @@
         <v>1851.0793671875001</v>
       </c>
       <c r="E247" s="5">
-        <f>(D247/C247)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.65416718018972564</v>
       </c>
     </row>
@@ -9266,7 +9266,7 @@
         <v>1851.0793671875001</v>
       </c>
       <c r="E248" s="5">
-        <f>(D248/C248)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.65416718018972564</v>
       </c>
     </row>
@@ -9284,7 +9284,7 @@
         <v>1091.839134765625</v>
       </c>
       <c r="E249" s="5">
-        <f>(D249/C249)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.7882647131520939</v>
       </c>
     </row>
@@ -9302,7 +9302,7 @@
         <v>139241.81425</v>
       </c>
       <c r="E250" s="5">
-        <f>(D250/C250)-1</f>
+        <f t="shared" si="3"/>
         <v>1.4502288182814587</v>
       </c>
     </row>
@@ -9320,7 +9320,7 @@
         <v>138748.16125</v>
       </c>
       <c r="E251" s="5">
-        <f>(D251/C251)-1</f>
+        <f t="shared" si="3"/>
         <v>1.4666072814131037</v>
       </c>
     </row>
@@ -9338,7 +9338,7 @@
         <v>138471.68724999999</v>
       </c>
       <c r="E252" s="5">
-        <f>(D252/C252)-1</f>
+        <f t="shared" si="3"/>
         <v>1.4739329177617364</v>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
         <v>138471.31849999999</v>
       </c>
       <c r="E253" s="5">
-        <f>(D253/C253)-1</f>
+        <f t="shared" si="3"/>
         <v>1.4739263296802196</v>
       </c>
     </row>
@@ -9374,7 +9374,7 @@
         <v>23.251758117675781</v>
       </c>
       <c r="E254" s="5">
-        <f>(D254/C254)-1</f>
+        <f t="shared" si="3"/>
         <v>-0.87891311192334043</v>
       </c>
     </row>
@@ -9392,7 +9392,7 @@
         <v>253.22912353515619</v>
       </c>
       <c r="E255" s="5">
-        <f>(D255/C255)-1</f>
+        <f t="shared" si="3"/>
         <v>1.9344656171073593</v>
       </c>
     </row>
@@ -9410,7 +9410,7 @@
         <v>142.54219946289061</v>
       </c>
       <c r="E256" s="5">
-        <f>(D256/C256)-1</f>
+        <f t="shared" si="3"/>
         <v>0.86497154258648745</v>
       </c>
     </row>
@@ -9428,7 +9428,7 @@
         <v>27.273954559326171</v>
       </c>
       <c r="E257" s="5">
-        <f>(D257/C257)-1</f>
+        <f t="shared" si="3"/>
         <v>17.08737619160831</v>
       </c>
     </row>
@@ -9446,7 +9446,7 @@
         <v>26.787793334960941</v>
       </c>
       <c r="E258" s="5">
-        <f>(D258/C258)-1</f>
+        <f t="shared" ref="E258:E321" si="4">(D258/C258)-1</f>
         <v>51.742258978068399</v>
       </c>
     </row>
@@ -9464,7 +9464,7 @@
         <v>83.412978515624999</v>
       </c>
       <c r="E259" s="5">
-        <f>(D259/C259)-1</f>
+        <f t="shared" si="4"/>
         <v>8.9828831580766177</v>
       </c>
     </row>
@@ -9482,7 +9482,7 @@
         <v>261.12446435546872</v>
       </c>
       <c r="E260" s="5">
-        <f>(D260/C260)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.52519086619825028</v>
       </c>
     </row>
@@ -9500,7 +9500,7 @@
         <v>229.32300341796881</v>
       </c>
       <c r="E261" s="5">
-        <f>(D261/C261)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.58301625670172064</v>
       </c>
     </row>
@@ -9518,7 +9518,7 @@
         <v>105.6209544677734</v>
       </c>
       <c r="E262" s="5">
-        <f>(D262/C262)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.8079467811415455</v>
       </c>
     </row>
@@ -9536,7 +9536,7 @@
         <v>232.52627416992189</v>
       </c>
       <c r="E263" s="5">
-        <f>(D263/C263)-1</f>
+        <f t="shared" si="4"/>
         <v>7.4491716812105064</v>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
         <v>172.70583422851561</v>
       </c>
       <c r="E264" s="5">
-        <f>(D264/C264)-1</f>
+        <f t="shared" si="4"/>
         <v>5.5096844484676417</v>
       </c>
     </row>
@@ -9572,7 +9572,7 @@
         <v>66.111624633789063</v>
       </c>
       <c r="E265" s="5">
-        <f>(D265/C265)-1</f>
+        <f t="shared" si="4"/>
         <v>1.6243623696004232</v>
       </c>
     </row>
@@ -9590,7 +9590,7 @@
         <v>121.6620620117187</v>
       </c>
       <c r="E266" s="5">
-        <f>(D266/C266)-1</f>
+        <f t="shared" si="4"/>
         <v>1.3353391522919891</v>
       </c>
     </row>
@@ -9608,7 +9608,7 @@
         <v>121.6620620117187</v>
       </c>
       <c r="E267" s="5">
-        <f>(D267/C267)-1</f>
+        <f t="shared" si="4"/>
         <v>1.3353391522919891</v>
       </c>
     </row>
@@ -9626,7 +9626,7 @@
         <v>0.37099200630187978</v>
       </c>
       <c r="E268" s="5">
-        <f>(D268/C268)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.87577699437405665</v>
       </c>
     </row>
@@ -9644,7 +9644,7 @@
         <v>19.64275253295898</v>
       </c>
       <c r="E269" s="5">
-        <f>(D269/C269)-1</f>
+        <f t="shared" si="4"/>
         <v>0.20350416529069237</v>
       </c>
     </row>
@@ -9662,7 +9662,7 @@
         <v>0.31397439765930168</v>
       </c>
       <c r="E270" s="5">
-        <f>(D270/C270)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.39643522172375689</v>
       </c>
     </row>
@@ -9680,7 +9680,7 @@
         <v>19.22824188232422</v>
       </c>
       <c r="E271" s="5">
-        <f>(D271/C271)-1</f>
+        <f t="shared" si="4"/>
         <v>0.31035238156508549</v>
       </c>
     </row>
@@ -9698,7 +9698,7 @@
         <v>2.4694094123840329</v>
       </c>
       <c r="E272" s="5">
-        <f>(D272/C272)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.78408968870142759</v>
       </c>
     </row>
@@ -9716,7 +9716,7 @@
         <v>16.60118441772461</v>
       </c>
       <c r="E273" s="5">
-        <f>(D273/C273)-1</f>
+        <f t="shared" si="4"/>
         <v>21.67301887151681</v>
       </c>
     </row>
@@ -9734,7 +9734,7 @@
         <v>101.6483142089844</v>
       </c>
       <c r="E274" s="5">
-        <f>(D274/C274)-1</f>
+        <f t="shared" si="4"/>
         <v>2.1001398123411219</v>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
         <v>100.66967187500001</v>
       </c>
       <c r="E275" s="5">
-        <f>(D275/C275)-1</f>
+        <f t="shared" si="4"/>
         <v>2.0796851434611163</v>
       </c>
     </row>
@@ -9770,7 +9770,7 @@
         <v>4.0763809051513666</v>
       </c>
       <c r="E276" s="5">
-        <f>(D276/C276)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.48483711137001229</v>
       </c>
     </row>
@@ -9788,7 +9788,7 @@
         <v>89.036286376953115</v>
       </c>
       <c r="E277" s="5">
-        <f>(D277/C277)-1</f>
+        <f t="shared" si="4"/>
         <v>3.7429104475670858</v>
       </c>
     </row>
@@ -9806,7 +9806,7 @@
         <v>2200.7571562500002</v>
       </c>
       <c r="E278" s="5">
-        <f>(D278/C278)-1</f>
+        <f t="shared" si="4"/>
         <v>6.9063412292613036E-2</v>
       </c>
     </row>
@@ -9824,7 +9824,7 @@
         <v>64.98731884765624</v>
       </c>
       <c r="E279" s="5">
-        <f>(D279/C279)-1</f>
+        <f t="shared" si="4"/>
         <v>0.18636326681690019</v>
       </c>
     </row>
@@ -9842,7 +9842,7 @@
         <v>37.825233459472663</v>
       </c>
       <c r="E280" s="5">
-        <f>(D280/C280)-1</f>
+        <f t="shared" si="4"/>
         <v>3.4806540541196487</v>
       </c>
     </row>
@@ -9860,7 +9860,7 @@
         <v>27.16209078979492</v>
       </c>
       <c r="E281" s="5">
-        <f>(D281/C281)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.41381041831216037</v>
       </c>
     </row>
@@ -9878,7 +9878,7 @@
         <v>24.38776739501953</v>
       </c>
       <c r="E282" s="5">
-        <f>(D282/C282)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.444109105113353</v>
       </c>
     </row>
@@ -9896,7 +9896,7 @@
         <v>685.8949931640625</v>
       </c>
       <c r="E283" s="5">
-        <f>(D283/C283)-1</f>
+        <f t="shared" si="4"/>
         <v>0.28285311526490875</v>
       </c>
     </row>
@@ -9914,7 +9914,7 @@
         <v>521.71349218749992</v>
       </c>
       <c r="E284" s="5">
-        <f>(D284/C284)-1</f>
+        <f t="shared" si="4"/>
         <v>0.16759877936265988</v>
       </c>
     </row>
@@ -9932,7 +9932,7 @@
         <v>164.18151538085939</v>
       </c>
       <c r="E285" s="5">
-        <f>(D285/C285)-1</f>
+        <f t="shared" si="4"/>
         <v>0.86914633899634675</v>
       </c>
     </row>
@@ -9950,7 +9950,7 @@
         <v>164.0229240722656</v>
       </c>
       <c r="E286" s="5">
-        <f>(D286/C286)-1</f>
+        <f t="shared" si="4"/>
         <v>0.86751092252695372</v>
       </c>
     </row>
@@ -9968,7 +9968,7 @@
         <v>281.32787353515619</v>
       </c>
       <c r="E287" s="5">
-        <f>(D287/C287)-1</f>
+        <f t="shared" si="4"/>
         <v>-6.9149196215170461E-2</v>
       </c>
     </row>
@@ -9986,7 +9986,7 @@
         <v>271.24359814453118</v>
       </c>
       <c r="E288" s="5">
-        <f>(D288/C288)-1</f>
+        <f t="shared" si="4"/>
         <v>0.23165516176512124</v>
       </c>
     </row>
@@ -10004,7 +10004,7 @@
         <v>4.02965291595459</v>
       </c>
       <c r="E289" s="5">
-        <f>(D289/C289)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.66610712703484309</v>
       </c>
     </row>
@@ -10022,7 +10022,7 @@
         <v>3.080932807922363</v>
       </c>
       <c r="E290" s="5">
-        <f>(D290/C290)-1</f>
+        <f t="shared" si="4"/>
         <v>-5.0325871425201063E-2</v>
       </c>
     </row>
@@ -10040,7 +10040,7 @@
         <v>267.21390966796872</v>
       </c>
       <c r="E291" s="5">
-        <f>(D291/C291)-1</f>
+        <f t="shared" si="4"/>
         <v>0.28370590093481174</v>
       </c>
     </row>
@@ -10058,7 +10058,7 @@
         <v>11.579764602661131</v>
       </c>
       <c r="E292" s="5">
-        <f>(D292/C292)-1</f>
+        <f t="shared" si="4"/>
         <v>1.4369217144368722</v>
       </c>
     </row>
@@ -10076,7 +10076,7 @@
         <v>6.6582210311889636</v>
       </c>
       <c r="E293" s="5">
-        <f>(D293/C293)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.95182763118765068</v>
       </c>
     </row>
@@ -10094,7 +10094,7 @@
         <v>6.06803197479248</v>
       </c>
       <c r="E294" s="5">
-        <f>(D294/C294)-1</f>
+        <f t="shared" si="4"/>
         <v>5.746005530619767</v>
       </c>
     </row>
@@ -10112,7 +10112,7 @@
         <v>45.442085205078122</v>
       </c>
       <c r="E295" s="5">
-        <f>(D295/C295)-1</f>
+        <f t="shared" si="4"/>
         <v>5.4649043689758869E-2</v>
       </c>
     </row>
@@ -10130,7 +10130,7 @@
         <v>132.13149389648439</v>
       </c>
       <c r="E296" s="5">
-        <f>(D296/C296)-1</f>
+        <f t="shared" si="4"/>
         <v>45.215982475160679</v>
       </c>
     </row>
@@ -10148,7 +10148,7 @@
         <v>10.084279891967769</v>
       </c>
       <c r="E297" s="5">
-        <f>(D297/C297)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.87702052700232114</v>
       </c>
     </row>
@@ -10166,7 +10166,7 @@
         <v>878.7076269531251</v>
       </c>
       <c r="E298" s="5">
-        <f>(D298/C298)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.12908643977142842</v>
       </c>
     </row>
@@ -10184,7 +10184,7 @@
         <v>835.265189453125</v>
       </c>
       <c r="E299" s="5">
-        <f>(D299/C299)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.16699840907006802</v>
       </c>
     </row>
@@ -10202,7 +10202,7 @@
         <v>829.5643720703124</v>
       </c>
       <c r="E300" s="5">
-        <f>(D300/C300)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.17268377703397542</v>
       </c>
     </row>
@@ -10220,7 +10220,7 @@
         <v>43.442502319335937</v>
       </c>
       <c r="E301" s="5">
-        <f>(D301/C301)-1</f>
+        <f t="shared" si="4"/>
         <v>5.9709883533650947</v>
       </c>
     </row>
@@ -10238,7 +10238,7 @@
         <v>43.337152893066403</v>
       </c>
       <c r="E302" s="5">
-        <f>(D302/C302)-1</f>
+        <f t="shared" si="4"/>
         <v>6.1057326555717264</v>
       </c>
     </row>
@@ -10256,7 +10256,7 @@
         <v>133.21086547851559</v>
       </c>
       <c r="E303" s="5">
-        <f>(D303/C303)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.14530785028121329</v>
       </c>
     </row>
@@ -10274,7 +10274,7 @@
         <v>130.09783764648441</v>
       </c>
       <c r="E304" s="5">
-        <f>(D304/C304)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.14177823308605841</v>
       </c>
     </row>
@@ -10292,7 +10292,7 @@
         <v>130.09783764648441</v>
       </c>
       <c r="E305" s="5">
-        <f>(D305/C305)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.14177823308605841</v>
       </c>
     </row>
@@ -10310,7 +10310,7 @@
         <v>3.1130287322998051</v>
       </c>
       <c r="E306" s="5">
-        <f>(D306/C306)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.27066309015303391</v>
       </c>
     </row>
@@ -10328,7 +10328,7 @@
         <v>1.742057577133179</v>
       </c>
       <c r="E307" s="5">
-        <f>(D307/C307)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.17351856099574015</v>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
         <v>0.638616021156311</v>
       </c>
       <c r="E308" s="5">
-        <f>(D308/C308)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.12012121637322815</v>
       </c>
     </row>
@@ -10364,7 +10364,7 @@
         <v>914.71571874999995</v>
       </c>
       <c r="E309" s="5">
-        <f>(D309/C309)-1</f>
+        <f t="shared" si="4"/>
         <v>0.63965983200004595</v>
       </c>
     </row>
@@ -10382,7 +10382,7 @@
         <v>5.0459629364013674</v>
       </c>
       <c r="E310" s="5">
-        <f>(D310/C310)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.7091060429598437</v>
       </c>
     </row>
@@ -10400,7 +10400,7 @@
         <v>0.6072751970291137</v>
       </c>
       <c r="E311" s="5">
-        <f>(D311/C311)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.95813079080886687</v>
       </c>
     </row>
@@ -10418,7 +10418,7 @@
         <v>2.668782436370849</v>
       </c>
       <c r="E312" s="5">
-        <f>(D312/C312)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.30713369428037562</v>
       </c>
     </row>
@@ -10436,7 +10436,7 @@
         <v>2.668782436370849</v>
       </c>
       <c r="E313" s="5">
-        <f>(D313/C313)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.30713369428037562</v>
       </c>
     </row>
@@ -10454,7 +10454,7 @@
         <v>4.2610268859863281</v>
       </c>
       <c r="E314" s="5">
-        <f>(D314/C314)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.96028147786285378</v>
       </c>
     </row>
@@ -10472,7 +10472,7 @@
         <v>2.8574879531860349</v>
       </c>
       <c r="E315" s="5">
-        <f>(D315/C315)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.97307363340988617</v>
       </c>
     </row>
@@ -10490,7 +10490,7 @@
         <v>0.46463681602478019</v>
       </c>
       <c r="E316" s="5">
-        <f>(D316/C316)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.99549178168189234</v>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
         <v>2.3928512496948242</v>
       </c>
       <c r="E317" s="5">
-        <f>(D317/C317)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.21748544762914934</v>
       </c>
     </row>
@@ -10526,7 +10526,7 @@
         <v>1.435068700790405</v>
       </c>
       <c r="E318" s="5">
-        <f>(D318/C318)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.4169468570306728</v>
       </c>
     </row>
@@ -10544,7 +10544,7 @@
         <v>0.74085119342803951</v>
       </c>
       <c r="E319" s="5">
-        <f>(D319/C319)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.36039783007162274</v>
       </c>
     </row>
@@ -10562,7 +10562,7 @@
         <v>0.74085119342803951</v>
       </c>
       <c r="E320" s="5">
-        <f>(D320/C320)-1</f>
+        <f t="shared" si="4"/>
         <v>-0.36039783007162274</v>
       </c>
     </row>
@@ -10580,7 +10580,7 @@
         <v>646.08220800781248</v>
       </c>
       <c r="E321" s="5">
-        <f>(D321/C321)-1</f>
+        <f t="shared" si="4"/>
         <v>0.54508123560115496</v>
       </c>
     </row>
@@ -10598,7 +10598,7 @@
         <v>2.4295727539062502</v>
       </c>
       <c r="E322" s="5">
-        <f>(D322/C322)-1</f>
+        <f t="shared" ref="E322:E385" si="5">(D322/C322)-1</f>
         <v>2.4530974911971981E-2</v>
       </c>
     </row>
@@ -10616,7 +10616,7 @@
         <v>2.4295727539062502</v>
       </c>
       <c r="E323" s="5">
-        <f>(D323/C323)-1</f>
+        <f t="shared" si="5"/>
         <v>2.4530974911971981E-2</v>
       </c>
     </row>
@@ -10634,7 +10634,7 @@
         <v>464.82426904296881</v>
       </c>
       <c r="E324" s="5">
-        <f>(D324/C324)-1</f>
+        <f t="shared" si="5"/>
         <v>0.59227181840748511</v>
       </c>
     </row>
@@ -10652,7 +10652,7 @@
         <v>177.22354028320311</v>
       </c>
       <c r="E325" s="5">
-        <f>(D325/C325)-1</f>
+        <f t="shared" si="5"/>
         <v>0.44272084685259272</v>
       </c>
     </row>
@@ -10670,7 +10670,7 @@
         <v>2.8610752983093271</v>
       </c>
       <c r="E326" s="5">
-        <f>(D326/C326)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.88356738758670861</v>
       </c>
     </row>
@@ -10688,7 +10688,7 @@
         <v>2278.2273828124999</v>
       </c>
       <c r="E327" s="5">
-        <f>(D327/C327)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.62070624925934381</v>
       </c>
     </row>
@@ -10706,7 +10706,7 @@
         <v>2278.2273828124999</v>
       </c>
       <c r="E328" s="5">
-        <f>(D328/C328)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.62070624925934381</v>
       </c>
     </row>
@@ -10724,7 +10724,7 @@
         <v>65.776976806640619</v>
       </c>
       <c r="E329" s="5">
-        <f>(D329/C329)-1</f>
+        <f t="shared" si="5"/>
         <v>0.67647441988822865</v>
       </c>
     </row>
@@ -10742,7 +10742,7 @@
         <v>2104.6602148437501</v>
       </c>
       <c r="E330" s="5">
-        <f>(D330/C330)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.64220935457156259</v>
       </c>
     </row>
@@ -10760,7 +10760,7 @@
         <v>2067.6100585937502</v>
       </c>
       <c r="E331" s="5">
-        <f>(D331/C331)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.64834107997511703</v>
       </c>
     </row>
@@ -10778,7 +10778,7 @@
         <v>822.41079492187498</v>
       </c>
       <c r="E332" s="5">
-        <f>(D332/C332)-1</f>
+        <f t="shared" si="5"/>
         <v>3.0941421029091476</v>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
         <v>811.84973730468744</v>
       </c>
       <c r="E333" s="5">
-        <f>(D333/C333)-1</f>
+        <f t="shared" si="5"/>
         <v>3.3448346693390958</v>
       </c>
     </row>
@@ -10814,7 +10814,7 @@
         <v>4.050703895568847</v>
       </c>
       <c r="E334" s="5">
-        <f>(D334/C334)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.54762472827927955</v>
       </c>
     </row>
@@ -10832,7 +10832,7 @@
         <v>6.2743906326293946</v>
       </c>
       <c r="E335" s="5">
-        <f>(D335/C335)-1</f>
+        <f t="shared" si="5"/>
         <v>0.30263263907434435</v>
       </c>
     </row>
@@ -10850,7 +10850,7 @@
         <v>996.934177734375</v>
       </c>
       <c r="E336" s="5">
-        <f>(D336/C336)-1</f>
+        <f t="shared" si="5"/>
         <v>0.47224578489670699</v>
       </c>
     </row>
@@ -10868,7 +10868,7 @@
         <v>944.36045312499994</v>
       </c>
       <c r="E337" s="5">
-        <f>(D337/C337)-1</f>
+        <f t="shared" si="5"/>
         <v>0.54935867764967972</v>
       </c>
     </row>
@@ -10886,7 +10886,7 @@
         <v>2.316953433990478</v>
       </c>
       <c r="E338" s="5">
-        <f>(D338/C338)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.94005372675669197</v>
       </c>
     </row>
@@ -10904,7 +10904,7 @@
         <v>122.36722436523441</v>
       </c>
       <c r="E339" s="5">
-        <f>(D339/C339)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.30370107821386538</v>
       </c>
     </row>
@@ -10922,7 +10922,7 @@
         <v>18.523639495849611</v>
       </c>
       <c r="E340" s="5">
-        <f>(D340/C340)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.69171044623551869</v>
       </c>
     </row>
@@ -10940,7 +10940,7 @@
         <v>6.0385792388916011</v>
       </c>
       <c r="E341" s="5">
-        <f>(D341/C341)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.33565330998497145</v>
       </c>
     </row>
@@ -10958,7 +10958,7 @@
         <v>16.61987579345703</v>
       </c>
       <c r="E342" s="5">
-        <f>(D342/C342)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.67364847252879101</v>
       </c>
     </row>
@@ -10976,7 +10976,7 @@
         <v>10.64916960144043</v>
       </c>
       <c r="E343" s="5">
-        <f>(D343/C343)-1</f>
+        <f t="shared" si="5"/>
         <v>0.4811908314009723</v>
       </c>
     </row>
@@ -10994,7 +10994,7 @@
         <v>64.083161132812492</v>
       </c>
       <c r="E344" s="5">
-        <f>(D344/C344)-1</f>
+        <f t="shared" si="5"/>
         <v>0.48755582429722932</v>
       </c>
     </row>
@@ -11012,7 +11012,7 @@
         <v>1.8269231929779051</v>
       </c>
       <c r="E345" s="5">
-        <f>(D345/C345)-1</f>
+        <f t="shared" si="5"/>
         <v>-2.9344577973557939E-3</v>
       </c>
     </row>
@@ -11030,7 +11030,7 @@
         <v>30.584751586914059</v>
       </c>
       <c r="E346" s="5">
-        <f>(D346/C346)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.99350465628990769</v>
       </c>
     </row>
@@ -11048,7 +11048,7 @@
         <v>6.123444854736328</v>
       </c>
       <c r="E347" s="5">
-        <f>(D347/C347)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.90188831085292598</v>
       </c>
     </row>
@@ -11066,7 +11066,7 @@
         <v>1.661911956787109</v>
       </c>
       <c r="E348" s="5">
-        <f>(D348/C348)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.3217239585392585</v>
       </c>
     </row>
@@ -11084,7 +11084,7 @@
         <v>35.388105651855469</v>
       </c>
       <c r="E349" s="5">
-        <f>(D349/C349)-1</f>
+        <f t="shared" si="5"/>
         <v>103.23595184640786</v>
       </c>
     </row>
@@ -11102,7 +11102,7 @@
         <v>65.91507800292969</v>
       </c>
       <c r="E350" s="5">
-        <f>(D350/C350)-1</f>
+        <f t="shared" si="5"/>
         <v>0.49026974727572936</v>
       </c>
     </row>
@@ -11120,7 +11120,7 @@
         <v>107.6521547851562</v>
       </c>
       <c r="E351" s="5">
-        <f>(D351/C351)-1</f>
+        <f t="shared" si="5"/>
         <v>0.34751824758736105</v>
       </c>
     </row>
@@ -11138,7 +11138,7 @@
         <v>3131.8946953125001</v>
       </c>
       <c r="E352" s="5">
-        <f>(D352/C352)-1</f>
+        <f t="shared" si="5"/>
         <v>0.12871791904719321</v>
       </c>
     </row>
@@ -11156,7 +11156,7 @@
         <v>3132.4337617187498</v>
       </c>
       <c r="E353" s="5">
-        <f>(D353/C353)-1</f>
+        <f t="shared" si="5"/>
         <v>0.1244299743576982</v>
       </c>
     </row>
@@ -11174,7 +11174,7 @@
         <v>62.380090698242178</v>
       </c>
       <c r="E354" s="5">
-        <f>(D354/C354)-1</f>
+        <f t="shared" si="5"/>
         <v>0.12681206756964758</v>
       </c>
     </row>
@@ -11192,7 +11192,7 @@
         <v>3683.75465234375</v>
       </c>
       <c r="E355" s="5">
-        <f>(D355/C355)-1</f>
+        <f t="shared" si="5"/>
         <v>0.10622335997357557</v>
       </c>
     </row>
@@ -11210,7 +11210,7 @@
         <v>233.60384521484369</v>
       </c>
       <c r="E356" s="5">
-        <f>(D356/C356)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.31449845584267855</v>
       </c>
     </row>
@@ -11228,7 +11228,7 @@
         <v>206.612814453125</v>
       </c>
       <c r="E357" s="5">
-        <f>(D357/C357)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.1975640454357005</v>
       </c>
     </row>
@@ -11246,7 +11246,7 @@
         <v>116.44004345703119</v>
       </c>
       <c r="E358" s="5">
-        <f>(D358/C358)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.41690035150704363</v>
       </c>
     </row>
@@ -11264,7 +11264,7 @@
         <v>39.978304931640622</v>
       </c>
       <c r="E359" s="5">
-        <f>(D359/C359)-1</f>
+        <f t="shared" si="5"/>
         <v>1.35918663808381</v>
       </c>
     </row>
@@ -11282,7 +11282,7 @@
         <v>34.376891601562498</v>
       </c>
       <c r="E360" s="5">
-        <f>(D360/C360)-1</f>
+        <f t="shared" si="5"/>
         <v>1.9141849718187327</v>
       </c>
     </row>
@@ -11300,7 +11300,7 @@
         <v>5.5760190048217773</v>
       </c>
       <c r="E361" s="5">
-        <f>(D361/C361)-1</f>
+        <f t="shared" si="5"/>
         <v>8.2848293941386819E-2</v>
       </c>
     </row>
@@ -11318,7 +11318,7 @@
         <v>50.194462463378898</v>
       </c>
       <c r="E362" s="5">
-        <f>(D362/C362)-1</f>
+        <f t="shared" si="5"/>
         <v>0.22891005352907223</v>
       </c>
     </row>
@@ -11336,7 +11336,7 @@
         <v>0.63427363204956055</v>
       </c>
       <c r="E363" s="5">
-        <f>(D363/C363)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.41627679730391998</v>
       </c>
     </row>
@@ -11354,7 +11354,7 @@
         <v>28.215028686523439</v>
       </c>
       <c r="E364" s="5">
-        <f>(D364/C364)-1</f>
+        <f t="shared" si="5"/>
         <v>-1.5130680959790532E-2</v>
       </c>
     </row>
@@ -11372,7 +11372,7 @@
         <v>20.40116217041016</v>
       </c>
       <c r="E365" s="5">
-        <f>(D365/C365)-1</f>
+        <f t="shared" si="5"/>
         <v>0.83635433952709004</v>
       </c>
     </row>
@@ -11390,7 +11390,7 @@
         <v>14.27139202880859</v>
       </c>
       <c r="E366" s="5">
-        <f>(D366/C366)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.15967591332560471</v>
       </c>
     </row>
@@ -11408,7 +11408,7 @@
         <v>0.95768802070617676</v>
       </c>
       <c r="E367" s="5">
-        <f>(D367/C367)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.55858774856831817</v>
       </c>
     </row>
@@ -11426,7 +11426,7 @@
         <v>13.313704345703121</v>
       </c>
       <c r="E368" s="5">
-        <f>(D368/C368)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.10125125926829925</v>
       </c>
     </row>
@@ -11444,7 +11444,7 @@
         <v>12.719645034790039</v>
       </c>
       <c r="E369" s="5">
-        <f>(D369/C369)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.80818718204041995</v>
       </c>
     </row>
@@ -11462,7 +11462,7 @@
         <v>9.1087497863769524</v>
       </c>
       <c r="E370" s="5">
-        <f>(D370/C370)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.81947285604250497</v>
       </c>
     </row>
@@ -11480,7 +11480,7 @@
         <v>3.6108945732116702</v>
       </c>
       <c r="E371" s="5">
-        <f>(D371/C371)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.77227525962944488</v>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
         <v>3.604286602020264</v>
       </c>
       <c r="E372" s="5">
-        <f>(D372/C372)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.77251266405239472</v>
       </c>
     </row>
@@ -11516,7 +11516,7 @@
         <v>317.71707421874999</v>
       </c>
       <c r="E373" s="5">
-        <f>(D373/C373)-1</f>
+        <f t="shared" si="5"/>
         <v>0.56162546899698595</v>
       </c>
     </row>
@@ -11534,7 +11534,7 @@
         <v>71.535375366210928</v>
       </c>
       <c r="E374" s="5">
-        <f>(D374/C374)-1</f>
+        <f t="shared" si="5"/>
         <v>0.94139019923226641</v>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
         <v>5.9967599639892573</v>
       </c>
       <c r="E375" s="5">
-        <f>(D375/C375)-1</f>
+        <f t="shared" si="5"/>
         <v>3.2784507438216037E-2</v>
       </c>
     </row>
@@ -11570,7 +11570,7 @@
         <v>65.535784057617178</v>
       </c>
       <c r="E376" s="5">
-        <f>(D376/C376)-1</f>
+        <f t="shared" si="5"/>
         <v>1.1148693872040294</v>
       </c>
     </row>
@@ -11588,7 +11588,7 @@
         <v>49.539891601562488</v>
       </c>
       <c r="E377" s="5">
-        <f>(D377/C377)-1</f>
+        <f t="shared" si="5"/>
         <v>6.6312663249322199</v>
       </c>
     </row>
@@ -11606,7 +11606,7 @@
         <v>1.571759963989257</v>
       </c>
       <c r="E378" s="5">
-        <f>(D378/C378)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.70091338788452251</v>
       </c>
     </row>
@@ -11624,7 +11624,7 @@
         <v>13.13604264831543</v>
       </c>
       <c r="E379" s="5">
-        <f>(D379/C379)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.29258973739765681</v>
       </c>
     </row>
@@ -11642,7 +11642,7 @@
         <v>117.99471362304691</v>
       </c>
       <c r="E380" s="5">
-        <f>(D380/C380)-1</f>
+        <f t="shared" si="5"/>
         <v>7.5942254173082313E-2</v>
       </c>
     </row>
@@ -11660,7 +11660,7 @@
         <v>99.864061157226544</v>
       </c>
       <c r="E381" s="5">
-        <f>(D381/C381)-1</f>
+        <f t="shared" si="5"/>
         <v>-4.8781380136941888E-4</v>
       </c>
     </row>
@@ -11678,7 +11678,7 @@
         <v>16.620723846435549</v>
       </c>
       <c r="E382" s="5">
-        <f>(D382/C382)-1</f>
+        <f t="shared" si="5"/>
         <v>1.8459656249782617</v>
       </c>
     </row>
@@ -11696,7 +11696,7 @@
         <v>1.359832019805908</v>
       </c>
       <c r="E383" s="5">
-        <f>(D383/C383)-1</f>
+        <f t="shared" si="5"/>
         <v>-0.64527663497954668</v>
       </c>
     </row>
@@ -11714,7 +11714,7 @@
         <v>125.7985727539062</v>
       </c>
       <c r="E384" s="5">
-        <f>(D384/C384)-1</f>
+        <f t="shared" si="5"/>
         <v>1.2550245268769742</v>
       </c>
     </row>
@@ -11732,7 +11732,7 @@
         <v>125.1402243652344</v>
       </c>
       <c r="E385" s="5">
-        <f>(D385/C385)-1</f>
+        <f t="shared" si="5"/>
         <v>1.2832890755785646</v>
       </c>
     </row>
@@ -11750,7 +11750,7 @@
         <v>30.361211303710931</v>
       </c>
       <c r="E386" s="5">
-        <f>(D386/C386)-1</f>
+        <f t="shared" ref="E386:E449" si="6">(D386/C386)-1</f>
         <v>2.1940677822009294</v>
       </c>
     </row>
@@ -11768,7 +11768,7 @@
         <v>7.7228637695312496</v>
       </c>
       <c r="E387" s="5">
-        <f>(D387/C387)-1</f>
+        <f t="shared" si="6"/>
         <v>-6.0798782710116961E-2</v>
       </c>
     </row>
@@ -11786,7 +11786,7 @@
         <v>87.056149291992185</v>
       </c>
       <c r="E388" s="5">
-        <f>(D388/C388)-1</f>
+        <f t="shared" si="6"/>
         <v>1.3478749064015778</v>
       </c>
     </row>
@@ -11804,7 +11804,7 @@
         <v>0.65834563159942627</v>
       </c>
       <c r="E389" s="5">
-        <f>(D389/C389)-1</f>
+        <f t="shared" si="6"/>
         <v>-0.3274638557570474</v>
       </c>
     </row>
@@ -11822,7 +11822,7 @@
         <v>0.28159519815444939</v>
       </c>
       <c r="E390" s="5">
-        <f>(D390/C390)-1</f>
+        <f t="shared" si="6"/>
         <v>-0.34390680765505721</v>
       </c>
     </row>
@@ -11840,7 +11840,7 @@
         <v>0.37675040531158438</v>
       </c>
       <c r="E391" s="5">
-        <f>(D391/C391)-1</f>
+        <f t="shared" si="6"/>
         <v>-0.31462542239115099</v>
       </c>
     </row>

</xml_diff>